<commit_message>
feat(report): export full member identity in operations XLSX
Sheet "Đội & thành viên" now includes Ngày sinh, Email, SĐT, CCCD, Khoa,
Facebook and Discord alongside the existing team/member columns, per the
organisers' request to have complete personal info in the export. The
report template header, styles and column widths grow to 15 columns to
match.

Also hardens the XLSX template parsing against XXE by routing worksheet
reads through defusedxml (new dependency) and adds the entity-rejection
test. The export endpoint stays admin/master_admin only and audited;
the prior test that asserted CCCD was withheld is updated to reflect the
deliberate decision to include it.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/backend/assets/vnutour-report-template.xlsx
+++ b/backend/assets/vnutour-report-template.xlsx
@@ -395,10 +395,17 @@
     <x:col min="2" max="2" width="28" hidden="0" customWidth="1"/>
     <x:col min="3" max="3" width="20" hidden="0" customWidth="1"/>
     <x:col min="4" max="4" width="16" hidden="0" customWidth="1"/>
-    <x:col min="5" max="5" width="16" hidden="0" customWidth="1"/>
-    <x:col min="6" max="6" width="28" hidden="0" customWidth="1"/>
-    <x:col min="7" max="7" width="24" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="14" hidden="0" customWidth="1"/>
+    <x:col min="6" max="6" width="16" hidden="0" customWidth="1"/>
+    <x:col min="7" max="7" width="28" hidden="0" customWidth="1"/>
     <x:col min="8" max="8" width="14" hidden="0" customWidth="1"/>
+    <x:col min="9" max="9" width="26" hidden="0" customWidth="1"/>
+    <x:col min="10" max="10" width="16" hidden="0" customWidth="1"/>
+    <x:col min="11" max="11" width="18" hidden="0" customWidth="1"/>
+    <x:col min="12" max="12" width="24" hidden="0" customWidth="1"/>
+    <x:col min="13" max="13" width="24" hidden="0" customWidth="1"/>
+    <x:col min="14" max="14" width="28" hidden="0" customWidth="1"/>
+    <x:col min="15" max="15" width="20" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1" ht="28" customHeight="1">
@@ -415,16 +422,37 @@
         <x:v>Đăng ký muộn</x:v>
       </x:c>
       <x:c r="E1" s="14" t="str">
+        <x:v>Đội trưởng</x:v>
+      </x:c>
+      <x:c r="F1" s="14" t="str">
         <x:v>MSSV</x:v>
       </x:c>
-      <x:c r="F1" s="14" t="str">
+      <x:c r="G1" s="14" t="str">
         <x:v>Họ tên</x:v>
       </x:c>
-      <x:c r="G1" s="14" t="str">
+      <x:c r="H1" s="14" t="str">
+        <x:v>Ngày sinh</x:v>
+      </x:c>
+      <x:c r="I1" s="14" t="str">
+        <x:v>Email</x:v>
+      </x:c>
+      <x:c r="J1" s="14" t="str">
+        <x:v>SĐT</x:v>
+      </x:c>
+      <x:c r="K1" s="14" t="str">
+        <x:v>CCCD</x:v>
+      </x:c>
+      <x:c r="L1" s="14" t="str">
         <x:v>Trường</x:v>
       </x:c>
-      <x:c r="H1" s="14" t="str">
-        <x:v>Đội trưởng</x:v>
+      <x:c r="M1" s="14" t="str">
+        <x:v>Khoa</x:v>
+      </x:c>
+      <x:c r="N1" s="14" t="str">
+        <x:v>Facebook</x:v>
+      </x:c>
+      <x:c r="O1" s="14" t="str">
+        <x:v>Discord</x:v>
       </x:c>
     </x:row>
     <x:row r="2" ht="22" customHeight="1">
@@ -436,6 +464,13 @@
       <x:c r="F2" s="18" t="str"/>
       <x:c r="G2" s="18" t="str"/>
       <x:c r="H2" s="18" t="str"/>
+      <x:c r="I2" s="18" t="str"/>
+      <x:c r="J2" s="18" t="str"/>
+      <x:c r="K2" s="18" t="str"/>
+      <x:c r="L2" s="18" t="str"/>
+      <x:c r="M2" s="18" t="str"/>
+      <x:c r="N2" s="18" t="str"/>
+      <x:c r="O2" s="18" t="str"/>
     </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>